<commit_message>
Rework sisimimi to follow supplied S-Chicken reference
</commit_message>
<xml_diff>
--- a/sisimimi/docs/PHAN_CONG.xlsx
+++ b/sisimimi/docs/PHAN_CONG.xlsx
@@ -512,14 +512,6 @@
           <t>SISIMIMI — PHÂN CÔNG VÀ ĐÁNH GIÁ NHÓM</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
-      <c r="H1" s="1" t="n"/>
-      <c r="I1" s="1" t="n"/>
     </row>
     <row r="2" ht="29" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -527,14 +519,6 @@
           <t>Mẫu nhiệm vụ gợi ý. Nhóm tự điền tên, mã sinh viên, tiến độ và điểm theo thực tế.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
     </row>
     <row r="3" ht="31" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -722,7 +706,7 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>js/script.js; toàn bộ website</t>
+          <t>js/products.js; js/cart.js; js/main.js; toàn bộ website</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr"/>

</xml_diff>